<commit_message>
Killing Floor 2 fix
Fixed Killing Floor 2 where the bootstrap would not start so it could install needed files to run a server.
</commit_message>
<xml_diff>
--- a/UGSM_Steam_Dedicated_Server_Tracker.xlsx
+++ b/UGSM_Steam_Dedicated_Server_Tracker.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\UGSMv2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F9CACC4-0D67-4595-9730-50C42428935C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5854915E-BA86-431B-951D-E5483B399DDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Steam Server Candidates" sheetId="1" r:id="rId1"/>
@@ -2144,6 +2144,9 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -2152,9 +2155,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2290,13 +2290,13 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>16</c:v>
+                  <c:v>18</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>50</c:v>
+                  <c:v>49</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>5</c:v>
+                  <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -3289,7 +3289,7 @@
       <c r="L11" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="M11" s="14" t="s">
+      <c r="M11" s="11" t="s">
         <v>667</v>
       </c>
       <c r="N11" s="4" t="s">
@@ -5378,7 +5378,7 @@
         <v>7</v>
       </c>
       <c r="I47" s="4" t="s">
-        <v>153</v>
+        <v>24</v>
       </c>
       <c r="J47" s="4" t="s">
         <v>292</v>
@@ -6836,7 +6836,7 @@
         <v>7</v>
       </c>
       <c r="I72" s="4" t="s">
-        <v>324</v>
+        <v>24</v>
       </c>
       <c r="J72" s="4" t="s">
         <v>325</v>
@@ -13332,16 +13332,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="27.95" customHeight="1">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="12" t="s">
         <v>560</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
       <c r="K1" s="2"/>
@@ -13439,7 +13439,7 @@
       </c>
       <c r="E4" s="2">
         <f>COUNTIF('Steam Server Candidates'!I2:I72,D4)</f>
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
@@ -13469,7 +13469,7 @@
       </c>
       <c r="B5" s="2">
         <f>COUNTIF('Steam Server Candidates'!I2:I72,"Done")</f>
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C5" s="2"/>
       <c r="D5" s="2" t="s">
@@ -13477,7 +13477,7 @@
       </c>
       <c r="E5" s="2">
         <f>COUNTIF('Steam Server Candidates'!I2:I72,D5)</f>
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
@@ -13507,7 +13507,7 @@
       </c>
       <c r="B6" s="2">
         <f>COUNTIF('Steam Server Candidates'!I2:I72,"Not Started")</f>
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C6" s="2"/>
       <c r="D6" s="2" t="s">
@@ -13515,7 +13515,7 @@
       </c>
       <c r="E6" s="2">
         <f>COUNTIF('Steam Server Candidates'!I2:I72,D6)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
@@ -13545,7 +13545,7 @@
       </c>
       <c r="B7" s="2">
         <f>COUNTIF('Steam Server Candidates'!I2:I72,"Later")</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C7" s="2"/>
       <c r="D7" s="2" t="s">
@@ -13765,16 +13765,16 @@
       <c r="Z13" s="2"/>
     </row>
     <row r="14" spans="1:26" ht="15">
-      <c r="A14" s="13" t="s">
+      <c r="A14" s="14" t="s">
         <v>570</v>
       </c>
-      <c r="B14" s="12"/>
-      <c r="C14" s="12"/>
-      <c r="D14" s="12"/>
-      <c r="E14" s="12"/>
-      <c r="F14" s="12"/>
-      <c r="G14" s="12"/>
-      <c r="H14" s="12"/>
+      <c r="B14" s="13"/>
+      <c r="C14" s="13"/>
+      <c r="D14" s="13"/>
+      <c r="E14" s="13"/>
+      <c r="F14" s="13"/>
+      <c r="G14" s="13"/>
+      <c r="H14" s="13"/>
       <c r="I14" s="2"/>
       <c r="J14" s="2"/>
       <c r="K14" s="2"/>

</xml_diff>